<commit_message>
api-autotest-tool v0.1 basic functions -> done.
</commit_message>
<xml_diff>
--- a/code/api-autotest-tool/case/case.xlsx
+++ b/code/api-autotest-tool/case/case.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sauro\Desktop\REPO\pw-z.github.io\code\api-autotest-tool\case\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2087\Desktop\REPO\pw-z.github.io\code\api-autotest-tool\case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F78635-8C61-4C36-BE0E-9EF16F1B6E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB021D82-2BB7-4435-A439-DA57587AA49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="353" windowWidth="20715" windowHeight="13424" tabRatio="780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="348" windowWidth="30936" windowHeight="17040" tabRatio="780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="test" sheetId="9" r:id="rId1"/>
@@ -73,9 +73,6 @@
     <t>ExpectedDQLData</t>
   </si>
   <si>
-    <t>sqlParameter1</t>
-  </si>
-  <si>
     <t>BASE</t>
   </si>
   <si>
@@ -97,10 +94,13 @@
     <t>application/x-www-form-urlencoded;charset=UTF-8</t>
   </si>
   <si>
-    <t>token</t>
-  </si>
-  <si>
-    <t>SELECT * FROM BASE_PARAM</t>
+    <t>token:token233</t>
+  </si>
+  <si>
+    <t>SELECT count(*) FROM BASE_PARAM</t>
+  </si>
+  <si>
+    <t>32</t>
   </si>
   <si>
     <t>信息获取</t>
@@ -222,7 +222,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -250,20 +250,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -273,7 +276,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -580,24 +583,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="7.46484375" customWidth="1"/>
-    <col min="2" max="2" width="12.86328125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" style="3" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="47.1328125" customWidth="1"/>
-    <col min="5" max="7" width="10.46484375" customWidth="1"/>
-    <col min="8" max="8" width="23.796875" customWidth="1"/>
+    <col min="4" max="4" width="47.109375" customWidth="1"/>
+    <col min="5" max="7" width="10.44140625" customWidth="1"/>
+    <col min="8" max="8" width="23.77734375" customWidth="1"/>
     <col min="9" max="9" width="5.33203125" customWidth="1"/>
-    <col min="10" max="10" width="10.46484375" customWidth="1"/>
+    <col min="10" max="10" width="10.44140625" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
     <col min="12" max="12" width="52.6640625" customWidth="1"/>
     <col min="13" max="13" width="43.33203125" customWidth="1"/>
-    <col min="14" max="18" width="26.46484375" customWidth="1"/>
+    <col min="14" max="16" width="26.44140625" customWidth="1"/>
+    <col min="17" max="17" width="26.44140625" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" ht="27" customHeight="1">
+    <row r="1" spans="1:17" s="1" customFormat="1" ht="27" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -649,54 +653,52 @@
       <c r="Q1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="6" t="s">
+    </row>
+    <row r="2" spans="1:17" s="2" customFormat="1" ht="64.95" customHeight="1">
+      <c r="A2" s="15" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" s="2" customFormat="1" ht="65" customHeight="1">
-      <c r="A2" s="14" t="s">
+      <c r="B2" s="10">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="9">
-        <v>1</v>
-      </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>20</v>
       </c>
       <c r="E2" s="7">
         <v>111</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H2"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>24</v>
       </c>
       <c r="M2" s="8"/>
       <c r="N2" s="7"/>
       <c r="O2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="Q2" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
     </row>
-    <row r="3" spans="1:18" ht="72" customHeight="1">
-      <c r="A3" s="15"/>
+    <row r="3" spans="1:17" ht="72" customHeight="1">
+      <c r="A3" s="16"/>
       <c r="B3" s="3">
         <v>2</v>
       </c>
@@ -711,9 +713,9 @@
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="I3" s="9"/>
       <c r="J3" s="7" t="s">
         <v>29</v>
       </c>
@@ -721,7 +723,7 @@
         <v>30</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="11" t="s">
@@ -730,7 +732,6 @@
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>